<commit_message>
Replace contextmeny with combobox  ProductsOrderingWidget.py -  Handle in CustomerRegistrationWidget.py
</commit_message>
<xml_diff>
--- a/Product specifications.xlsx
+++ b/Product specifications.xlsx
@@ -23,499 +23,499 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="165">
   <si>
-    <t>iqos iluma one moss green</t>
-  </si>
-  <si>
-    <t>iqos iluma one sunset red</t>
-  </si>
-  <si>
-    <t>iqos iluma one pebble gray</t>
-  </si>
-  <si>
-    <t>iqos iluma one azure blue</t>
-  </si>
-  <si>
-    <t>iqos iluma standard moss green</t>
-  </si>
-  <si>
-    <t>iqos 3 duo limited edition passion red</t>
-  </si>
-  <si>
-    <t>iqos iluma standard sunset red</t>
-  </si>
-  <si>
-    <t>iqos iluma standard pebble gray</t>
-  </si>
-  <si>
-    <t>iqos iluma standard azure blue</t>
-  </si>
-  <si>
-    <t>iqos iluma standard gold</t>
-  </si>
-  <si>
-    <t>iqos iluma standard oasis limited edition</t>
-  </si>
-  <si>
-    <t>iqos iluma prime gold</t>
-  </si>
-  <si>
-    <t>iqos iluma prime jade green</t>
-  </si>
-  <si>
-    <t>iqos iluma prime obsidian black</t>
-  </si>
-  <si>
-    <t>iqos iluma prime bronze taupe</t>
-  </si>
-  <si>
-    <t>iqos iluma standard neon limited edition</t>
-  </si>
-  <si>
-    <t>iqos originals duo slate</t>
-  </si>
-  <si>
-    <t>iqos originals duo tourquise</t>
-  </si>
-  <si>
-    <t>iqos originals duo scarlet red</t>
-  </si>
-  <si>
-    <t>iqos originals duo silver</t>
-  </si>
-  <si>
-    <t>iqos 3 duo gold</t>
-  </si>
-  <si>
-    <t>iqos 3 duo gray</t>
-  </si>
-  <si>
-    <t>iqos 3 duo white</t>
-  </si>
-  <si>
-    <t>iqos 3 duo blue</t>
-  </si>
-  <si>
-    <t>heets purple wave armania</t>
-  </si>
-  <si>
-    <t>heets turquoise armania</t>
-  </si>
-  <si>
-    <t>heets bronze armania</t>
-  </si>
-  <si>
-    <t>heets silver armania</t>
-  </si>
-  <si>
-    <t>heets yellow armania</t>
-  </si>
-  <si>
-    <t>heets amber armania</t>
-  </si>
-  <si>
-    <t>heets dimensions yugen armania</t>
-  </si>
-  <si>
-    <t>heets dimensions noor armania</t>
-  </si>
-  <si>
-    <t>heets satin fuse russian parliament</t>
-  </si>
-  <si>
-    <t>heets dimensions glaze russian</t>
-  </si>
-  <si>
-    <t>heets dimensions apricity russian</t>
-  </si>
-  <si>
-    <t>heets slate russian parliament</t>
-  </si>
-  <si>
-    <t>heets green zing russian parliament</t>
-  </si>
-  <si>
-    <t>heets purple wave russian parliament</t>
-  </si>
-  <si>
-    <t>heets summer breeze russian parliament</t>
-  </si>
-  <si>
-    <t>heets tropical swift russian parliament</t>
-  </si>
-  <si>
-    <t>heets ruby fuse russian parliament</t>
-  </si>
-  <si>
-    <t>heets amarello fuse russian parliament</t>
-  </si>
-  <si>
-    <t>heets teak russian parliament</t>
-  </si>
-  <si>
-    <t>heets gold russian parliament</t>
-  </si>
-  <si>
-    <t>heets sienna caps europian</t>
-  </si>
-  <si>
-    <t>heets turquoise europian</t>
-  </si>
-  <si>
-    <t>heets purple wave europian</t>
-  </si>
-  <si>
-    <t>heets bronze europian</t>
-  </si>
-  <si>
-    <t>heets yellow europian</t>
-  </si>
-  <si>
-    <t>heets amber europian</t>
-  </si>
-  <si>
-    <t>heets silver europian</t>
-  </si>
-  <si>
-    <t>heets teak europian</t>
-  </si>
-  <si>
-    <t>heets sienna europian</t>
-  </si>
-  <si>
-    <t>heets purple wave arabic</t>
-  </si>
-  <si>
-    <t>heets teak arabic</t>
-  </si>
-  <si>
-    <t>heets sienna arabic</t>
-  </si>
-  <si>
-    <t>heets turquoise arabic</t>
-  </si>
-  <si>
-    <t>heets bronze arabic</t>
-  </si>
-  <si>
-    <t>heets yellow arabic</t>
-  </si>
-  <si>
-    <t>heets amber arabic</t>
-  </si>
-  <si>
-    <t>heets silver arabic</t>
-  </si>
-  <si>
-    <t>terea oasis pearl japanies</t>
-  </si>
-  <si>
-    <t>terea bold regular japanies</t>
-  </si>
-  <si>
-    <t>terea regular japanies</t>
-  </si>
-  <si>
-    <t>terea fusion menthol japanies</t>
-  </si>
-  <si>
-    <t>terea warm regular japanies</t>
-  </si>
-  <si>
-    <t>terea black menthol japanies</t>
-  </si>
-  <si>
-    <t>terea tropical japanies</t>
-  </si>
-  <si>
-    <t>terea black purple menthol japanies</t>
-  </si>
-  <si>
-    <t>terea purple menthol japanies</t>
-  </si>
-  <si>
-    <t>terea bright menthol japanies</t>
-  </si>
-  <si>
-    <t>terea menthol japanies</t>
-  </si>
-  <si>
-    <t>terea yellow menthol japanies</t>
-  </si>
-  <si>
-    <t>terea balanced regular japanies</t>
-  </si>
-  <si>
-    <t>terea rich regular japanies</t>
-  </si>
-  <si>
-    <t>terea smoth regular japanies</t>
-  </si>
-  <si>
-    <t>terea yellow italy</t>
-  </si>
-  <si>
-    <t>terea sienna italy</t>
-  </si>
-  <si>
-    <t>terea bronze italy</t>
-  </si>
-  <si>
-    <t>terea amber italy</t>
-  </si>
-  <si>
-    <t>terea teak italy</t>
-  </si>
-  <si>
-    <t>fiit crisp armania</t>
-  </si>
-  <si>
-    <t>fiit sky regular armania</t>
-  </si>
-  <si>
-    <t>fiit regular armania</t>
-  </si>
-  <si>
-    <t>iluma ring set</t>
-  </si>
-  <si>
-    <t>iqos iluma standard silicone chartreuse</t>
-  </si>
-  <si>
-    <t>iqos iluma standard silicone bright coral</t>
-  </si>
-  <si>
-    <t>iqos iluma standard silicone tinted teal</t>
-  </si>
-  <si>
-    <t>iqos iluma standard silicone clarlet red</t>
-  </si>
-  <si>
-    <t>iqos iluma standard silicone new indigo</t>
-  </si>
-  <si>
-    <t>iqos iluma standard sleeve plus khaki</t>
-  </si>
-  <si>
-    <t>iqos iluma standard sleeve plus dark gray</t>
-  </si>
-  <si>
-    <t>iqos iluma standard sleeve dark green</t>
-  </si>
-  <si>
-    <t>os iluma prime silicone sleeve obsidian black</t>
-  </si>
-  <si>
-    <t>iqos iluma prime silicone sleeve citron yellow</t>
-  </si>
-  <si>
-    <t>iqos iluma prime silicone sleeve lake blue</t>
-  </si>
-  <si>
-    <t>iqos iluma prime silicone sleeve bright coral</t>
-  </si>
-  <si>
-    <t>iqos 3duo leather sleeve deep red</t>
-  </si>
-  <si>
-    <t>iqos 3duo leather sleeve cream</t>
-  </si>
-  <si>
     <t>cleaning pack frie quos</t>
   </si>
   <si>
-    <t>iqos cleaner 10ml</t>
-  </si>
-  <si>
-    <t>iqos cleaner 60ml</t>
-  </si>
-  <si>
-    <t>iqos lil solid 2 cap blue</t>
-  </si>
-  <si>
-    <t>iqos lil solid 2 cap black</t>
-  </si>
-  <si>
-    <t>iqos 3 duo folio leather white</t>
-  </si>
-  <si>
     <t>charging dock 2.4 plus</t>
   </si>
   <si>
-    <t>iqos 3 duo side door stellar blue</t>
-  </si>
-  <si>
-    <t>iqos 3 duo side door purple</t>
-  </si>
-  <si>
-    <t>iqos 3 duo side door white</t>
-  </si>
-  <si>
-    <t>iqos 3 duo side door yellow</t>
-  </si>
-  <si>
-    <t>iqos 3 duo side door green</t>
-  </si>
-  <si>
-    <t>iqos 3 duo side door bronze</t>
-  </si>
-  <si>
-    <t>iqos 3 duo side door light green</t>
-  </si>
-  <si>
-    <t>iqos 3 duo cap leaden</t>
-  </si>
-  <si>
-    <t>iqos 3 duo cap red</t>
-  </si>
-  <si>
-    <t>iqos 3 duo cap blue</t>
-  </si>
-  <si>
-    <t>iqos 3 duo silicone cover purple</t>
-  </si>
-  <si>
-    <t>iqos 3 duo silicone cover yellow</t>
-  </si>
-  <si>
-    <t>iqos 3 duo silicone cover magenta</t>
-  </si>
-  <si>
-    <t>iqos 3 duo silicone cover orange</t>
-  </si>
-  <si>
-    <t>iqos 3 duo folio red</t>
-  </si>
-  <si>
-    <t>iqos 3 duo sleeve red</t>
-  </si>
-  <si>
-    <t>mega pack iqos</t>
-  </si>
-  <si>
-    <t>charging iqos 3 duo</t>
-  </si>
-  <si>
-    <t>iqos 3 duo pocket charge gold</t>
-  </si>
-  <si>
-    <t>iqos 3 duo pocket charge black</t>
-  </si>
-  <si>
-    <t>iqos 3 duo pocket charge white</t>
-  </si>
-  <si>
-    <t>iqos 3 duo pocket charge stellar blue</t>
-  </si>
-  <si>
     <t>cleaning stick</t>
   </si>
   <si>
     <t>cleaner tools</t>
   </si>
   <si>
-    <t>iqos 3 duo holder gold</t>
-  </si>
-  <si>
-    <t>iqos 3 duo holder stellar blue</t>
-  </si>
-  <si>
-    <t>iqos 3 duo holder warm white</t>
-  </si>
-  <si>
-    <t>iqos 3 duo holder velvet gray</t>
-  </si>
-  <si>
-    <t>terea sienna indonesia</t>
-  </si>
-  <si>
-    <t>terea purple wave indonesia</t>
-  </si>
-  <si>
-    <t>terea green indonesia</t>
-  </si>
-  <si>
-    <t>terea bright wave indonesia</t>
-  </si>
-  <si>
-    <t>terea dimensions apricity indonesia</t>
-  </si>
-  <si>
-    <t>terea dimensions yugen indonesia</t>
-  </si>
-  <si>
-    <t>terea blue indonesia</t>
-  </si>
-  <si>
-    <t>terea bronze indonesia</t>
-  </si>
-  <si>
-    <t>terea black green indinesia</t>
-  </si>
-  <si>
-    <t>iqos iluma prime oasis limited edition</t>
-  </si>
-  <si>
-    <t>terea sienna europian</t>
-  </si>
-  <si>
-    <t>terea black yellow menthol japanies</t>
-  </si>
-  <si>
-    <t>heets dimensions amil europian</t>
-  </si>
-  <si>
-    <t>iqos lil solid2 blue</t>
-  </si>
-  <si>
-    <t>iqos lil solid2 black</t>
-  </si>
-  <si>
-    <t>terea ruby regular japanies</t>
-  </si>
-  <si>
-    <t>heets apricity arabic</t>
-  </si>
-  <si>
-    <t>heets sun pearl europain</t>
-  </si>
-  <si>
-    <t>heets sienna armania</t>
-  </si>
-  <si>
-    <t>terea purple wave europain</t>
-  </si>
-  <si>
-    <t>terea turquoise eruopain</t>
-  </si>
-  <si>
-    <t>terea yellow europain</t>
-  </si>
-  <si>
-    <t>iqos lil solid Ez mint</t>
-  </si>
-  <si>
-    <t>iqos lil solid Ez black</t>
-  </si>
-  <si>
-    <t>iqos lil solid Ez blue</t>
-  </si>
-  <si>
-    <t>iqos lil solid Ez white</t>
-  </si>
-  <si>
-    <t>heets</t>
-  </si>
-  <si>
     <t>acce</t>
   </si>
   <si>
-    <t>terea mint japanes</t>
-  </si>
-  <si>
-    <t>terea</t>
-  </si>
-  <si>
-    <t>iqos</t>
+    <t>fiit crisp Armenia</t>
+  </si>
+  <si>
+    <t>fiit sky regular Armenia</t>
+  </si>
+  <si>
+    <t>fiit regular Armenia</t>
+  </si>
+  <si>
+    <t>Heets purple wave Armenia</t>
+  </si>
+  <si>
+    <t>Heets turquoise Armenia</t>
+  </si>
+  <si>
+    <t>Heets bronze Armenia</t>
+  </si>
+  <si>
+    <t>Heets silver Armenia</t>
+  </si>
+  <si>
+    <t>Heets yellow Armenia</t>
+  </si>
+  <si>
+    <t>Heets amber Armenia</t>
+  </si>
+  <si>
+    <t>Heets dimensions yugen Armenia</t>
+  </si>
+  <si>
+    <t>Heets dimensions noor Armenia</t>
+  </si>
+  <si>
+    <t>Heets satin fuse Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets dimensions glaze Russian</t>
+  </si>
+  <si>
+    <t>Heets dimensions apricity Russian</t>
+  </si>
+  <si>
+    <t>Heets slate Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets green zing Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets purple wave Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets summer breeze Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets tropical swift Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets ruby fuse Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets amarello fuse Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets teak Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets gold Russian parliament</t>
+  </si>
+  <si>
+    <t>Heets sienna caps European</t>
+  </si>
+  <si>
+    <t>Heets turquoise European</t>
+  </si>
+  <si>
+    <t>Heets purple wave European</t>
+  </si>
+  <si>
+    <t>Heets bronze European</t>
+  </si>
+  <si>
+    <t>Heets yellow European</t>
+  </si>
+  <si>
+    <t>Heets amber European</t>
+  </si>
+  <si>
+    <t>Heets silver European</t>
+  </si>
+  <si>
+    <t>Heets teak European</t>
+  </si>
+  <si>
+    <t>Heets sienna European</t>
+  </si>
+  <si>
+    <t>Heets purple wave Arabic</t>
+  </si>
+  <si>
+    <t>Heets teak Arabic</t>
+  </si>
+  <si>
+    <t>Heets sienna Arabic</t>
+  </si>
+  <si>
+    <t>Heets turquoise Arabic</t>
+  </si>
+  <si>
+    <t>Heets bronze Arabic</t>
+  </si>
+  <si>
+    <t>Heets yellow Arabic</t>
+  </si>
+  <si>
+    <t>Heets amber Arabic</t>
+  </si>
+  <si>
+    <t>Heets silver Arabic</t>
+  </si>
+  <si>
+    <t>Heets</t>
+  </si>
+  <si>
+    <t>Heets dimensions amil European</t>
+  </si>
+  <si>
+    <t>Heets apricity Arabic</t>
+  </si>
+  <si>
+    <t>Heets sun pearl European</t>
+  </si>
+  <si>
+    <t>Heets sienna Armenia</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo limited edition passion red</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo gold</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo gray</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo white</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo blue</t>
+  </si>
+  <si>
+    <t>Iqos 3duo leather sleeve deep red</t>
+  </si>
+  <si>
+    <t>Iqos 3duo leather sleeve cream</t>
+  </si>
+  <si>
+    <t>Iqos cleaner 10ml</t>
+  </si>
+  <si>
+    <t>Iqos cleaner 60ml</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo folio leather white</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo side door stellar blue</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo side door purple</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo side door white</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo side door yellow</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo side door green</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo side door bronze</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo side door light green</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo cap leaden</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo cap red</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo cap blue</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo silicone cover purple</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo silicone cover yellow</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo silicone cover magenta</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo silicone cover orange</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo folio red</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo sleeve red</t>
+  </si>
+  <si>
+    <t>mega pack Iqos</t>
+  </si>
+  <si>
+    <t>charging Iqos 3 duo</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo pocket charge gold</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo pocket charge black</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo pocket charge white</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo pocket charge stellar blue</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo holder gold</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo holder stellar blue</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo holder warm white</t>
+  </si>
+  <si>
+    <t>Iqos 3 duo holder velvet gray</t>
+  </si>
+  <si>
+    <t>Iqos</t>
+  </si>
+  <si>
+    <t>Terea oasis pearl Japanese</t>
+  </si>
+  <si>
+    <t>Terea bold regular Japanese</t>
+  </si>
+  <si>
+    <t>Terea regular Japanese</t>
+  </si>
+  <si>
+    <t>Terea fusion menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea warm regular Japanese</t>
+  </si>
+  <si>
+    <t>Terea black menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea tropical Japanese</t>
+  </si>
+  <si>
+    <t>Terea black purple menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea purple menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea bright menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea yellow menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea balanced regular Japanese</t>
+  </si>
+  <si>
+    <t>Terea rich regular Japanese</t>
+  </si>
+  <si>
+    <t>Terea smoth regular Japanese</t>
+  </si>
+  <si>
+    <t>Terea yellow Italian</t>
+  </si>
+  <si>
+    <t>Terea sienna Italian</t>
+  </si>
+  <si>
+    <t>Terea bronze Italian</t>
+  </si>
+  <si>
+    <t>Terea amber Italian</t>
+  </si>
+  <si>
+    <t>Terea teak Italian</t>
+  </si>
+  <si>
+    <t>Terea mint Japanese</t>
+  </si>
+  <si>
+    <t>Terea sienna Indonesian</t>
+  </si>
+  <si>
+    <t>Terea</t>
+  </si>
+  <si>
+    <t>Terea purple wave Indonesian</t>
+  </si>
+  <si>
+    <t>Terea green Indonesian</t>
+  </si>
+  <si>
+    <t>Terea bright wave Indonesian</t>
+  </si>
+  <si>
+    <t>Terea dimensions apricity Indonesian</t>
+  </si>
+  <si>
+    <t>Terea dimensions yugen Indonesian</t>
+  </si>
+  <si>
+    <t>Terea blue Indonesian</t>
+  </si>
+  <si>
+    <t>Terea bronze Indonesian</t>
+  </si>
+  <si>
+    <t>Terea black green Indonesian</t>
+  </si>
+  <si>
+    <t>Terea sienna European</t>
+  </si>
+  <si>
+    <t>Terea black yellow menthol Japanese</t>
+  </si>
+  <si>
+    <t>Terea ruby regular Japanese</t>
+  </si>
+  <si>
+    <t>Terea purple wave European</t>
+  </si>
+  <si>
+    <t>Terea turquoise European</t>
+  </si>
+  <si>
+    <t>Terea yellow European</t>
+  </si>
+  <si>
+    <t>Iqos Iluma one moss green</t>
+  </si>
+  <si>
+    <t>Iqos Iluma one sunset red</t>
+  </si>
+  <si>
+    <t>Iqos Iluma one pebble gray</t>
+  </si>
+  <si>
+    <t>Iqos Iluma one azure blue</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard moss green</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard sunset red</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard pebble gray</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard azure blue</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard gold</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard oasis limited edition</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime gold</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime jade green</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime obsidian black</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime bronze taupe</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard neon limited edition</t>
+  </si>
+  <si>
+    <t>Iluma ring set</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard silicone chartreuse</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard silicone bright coral</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard silicone tinted teal</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard silicone clarlet red</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard silicone new indigo</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard sleeve plus khaki</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard sleeve plus dark gray</t>
+  </si>
+  <si>
+    <t>Iqos Iluma standard sleeve dark green</t>
+  </si>
+  <si>
+    <t>os Iluma prime silicone sleeve obsidian black</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime silicone sleeve citron yellow</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime silicone sleeve lake blue</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime silicone sleeve bright coral</t>
+  </si>
+  <si>
+    <t>Iqos Iluma prime oasis limited edition</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid 2 cap blue</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid 2 cap black</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid2 blue</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid2 black</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid Ez mint</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid Ez black</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid Ez blue</t>
+  </si>
+  <si>
+    <t>Iqos Lil solid Ez white</t>
+  </si>
+  <si>
+    <t>Iqos Originals duo slate</t>
+  </si>
+  <si>
+    <t>Iqos Originals duo tourquise</t>
+  </si>
+  <si>
+    <t>Iqos Originals duo scarlet red</t>
+  </si>
+  <si>
+    <t>Iqos Originals duo silver</t>
   </si>
 </sst>
 </file>
@@ -865,13 +865,13 @@
   <dimension ref="A1:D162"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" customWidth="1"/>
     <col min="2" max="2" width="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="B1" s="2">
         <v>1001</v>
@@ -879,7 +879,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="B2" s="2">
         <v>1002</v>
@@ -887,7 +887,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>126</v>
       </c>
       <c r="B3" s="2">
         <v>1003</v>
@@ -895,7 +895,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>127</v>
       </c>
       <c r="B4" s="2">
         <v>1004</v>
@@ -903,7 +903,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>128</v>
       </c>
       <c r="B5" s="2">
         <v>1005</v>
@@ -911,7 +911,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="B6" s="2">
         <v>1006</v>
@@ -919,7 +919,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>129</v>
       </c>
       <c r="B7" s="2">
         <v>1007</v>
@@ -927,7 +927,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>130</v>
       </c>
       <c r="B8" s="2">
         <v>1008</v>
@@ -935,7 +935,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>8</v>
+        <v>131</v>
       </c>
       <c r="B9" s="2">
         <v>1009</v>
@@ -943,7 +943,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>9</v>
+        <v>132</v>
       </c>
       <c r="B10" s="2">
         <v>1010</v>
@@ -951,7 +951,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="B11" s="2">
         <v>1011</v>
@@ -959,7 +959,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>11</v>
+        <v>134</v>
       </c>
       <c r="B12" s="2">
         <v>1012</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>12</v>
+        <v>135</v>
       </c>
       <c r="B13" s="2">
         <v>1013</v>
@@ -975,7 +975,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>136</v>
       </c>
       <c r="B14" s="2">
         <v>1014</v>
@@ -983,7 +983,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>14</v>
+        <v>137</v>
       </c>
       <c r="B15" s="2">
         <v>1015</v>
@@ -991,7 +991,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>15</v>
+        <v>138</v>
       </c>
       <c r="B16" s="2">
         <v>1016</v>
@@ -999,7 +999,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>16</v>
+        <v>161</v>
       </c>
       <c r="B17" s="2">
         <v>1017</v>
@@ -1007,7 +1007,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>17</v>
+        <v>162</v>
       </c>
       <c r="B18" s="2">
         <v>1018</v>
@@ -1015,7 +1015,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>18</v>
+        <v>163</v>
       </c>
       <c r="B19" s="2">
         <v>1019</v>
@@ -1023,7 +1023,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>164</v>
       </c>
       <c r="B20" s="2">
         <v>1020</v>
@@ -1031,7 +1031,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="B21" s="2">
         <v>1021</v>
@@ -1039,7 +1039,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="B22" s="2">
         <v>1022</v>
@@ -1047,7 +1047,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="B23" s="2">
         <v>1023</v>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="B24" s="2">
         <v>1024</v>
@@ -1063,7 +1063,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B25" s="2">
         <v>1025</v>
@@ -1071,7 +1071,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="B26" s="2">
         <v>1026</v>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="B27" s="2">
         <v>1027</v>
@@ -1087,7 +1087,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B28" s="2">
         <v>1028</v>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B29" s="2">
         <v>1029</v>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="B30" s="2">
         <v>1030</v>
@@ -1111,7 +1111,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="B31" s="2">
         <v>1031</v>
@@ -1119,7 +1119,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="B32" s="2">
         <v>1032</v>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B33" s="2">
         <v>1033</v>
@@ -1135,7 +1135,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B34" s="2">
         <v>1034</v>
@@ -1143,7 +1143,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B35" s="2">
         <v>1035</v>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B36" s="2">
         <v>1036</v>
@@ -1159,7 +1159,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="B37" s="2">
         <v>1037</v>
@@ -1167,7 +1167,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="B38" s="2">
         <v>1038</v>
@@ -1175,7 +1175,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B39" s="2">
         <v>1039</v>
@@ -1183,7 +1183,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="B40" s="2">
         <v>1040</v>
@@ -1191,7 +1191,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B41" s="2">
         <v>1041</v>
@@ -1199,7 +1199,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B42" s="2">
         <v>1042</v>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B43" s="2">
         <v>1043</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="B44" s="2">
         <v>1044</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="B45" s="2">
         <v>1045</v>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="B46" s="2">
         <v>1046</v>
@@ -1239,7 +1239,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="B47" s="2">
         <v>1047</v>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B48" s="2">
         <v>1048</v>
@@ -1255,7 +1255,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B49" s="2">
         <v>1049</v>
@@ -1263,7 +1263,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="B50" s="2">
         <v>1050</v>
@@ -1271,7 +1271,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="B51" s="2">
         <v>1051</v>
@@ -1279,7 +1279,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B52" s="2">
         <v>1052</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B53" s="2">
         <v>1053</v>
@@ -1295,7 +1295,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="B54" s="2">
         <v>1054</v>
@@ -1303,7 +1303,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="B55" s="2">
         <v>1055</v>
@@ -1311,7 +1311,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="B56" s="2">
         <v>1056</v>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="B57" s="2">
         <v>1057</v>
@@ -1327,7 +1327,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="B58" s="2">
         <v>1058</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="B59" s="2">
         <v>1059</v>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="B60" s="2">
         <v>1060</v>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="B61" s="2">
         <v>1061</v>
@@ -1359,7 +1359,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="B62" s="2">
         <v>1062</v>
@@ -1367,7 +1367,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="B63" s="2">
         <v>1063</v>
@@ -1375,7 +1375,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="B64" s="2">
         <v>1064</v>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="B65" s="2">
         <v>1065</v>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="B66" s="2">
         <v>1066</v>
@@ -1399,7 +1399,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="B67" s="2">
         <v>1067</v>
@@ -1407,7 +1407,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="B68" s="2">
         <v>1068</v>
@@ -1415,7 +1415,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="B69" s="2">
         <v>1069</v>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="B70" s="2">
         <v>1070</v>
@@ -1431,7 +1431,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="B71" s="2">
         <v>1071</v>
@@ -1439,7 +1439,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="B72" s="2">
         <v>1072</v>
@@ -1447,7 +1447,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="B73" s="2">
         <v>1073</v>
@@ -1455,7 +1455,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="B74" s="2">
         <v>1074</v>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="B75" s="2">
         <v>1075</v>
@@ -1471,7 +1471,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
       <c r="B76" s="2">
         <v>1076</v>
@@ -1479,7 +1479,7 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="B77" s="2">
         <v>1077</v>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="B78" s="2">
         <v>1078</v>
@@ -1495,7 +1495,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="B79" s="2">
         <v>1079</v>
@@ -1503,7 +1503,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="B80" s="2">
         <v>1080</v>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="B81" s="2">
         <v>1081</v>
@@ -1519,18 +1519,18 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>81</v>
+        <v>5</v>
       </c>
       <c r="B82" s="2">
         <v>1082</v>
       </c>
       <c r="D82" t="s">
-        <v>160</v>
+        <v>45</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>82</v>
+        <v>6</v>
       </c>
       <c r="B83" s="2">
         <v>1083</v>
@@ -1538,7 +1538,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="B84" s="2">
         <v>1084</v>
@@ -1546,40 +1546,40 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>84</v>
+        <v>139</v>
       </c>
       <c r="B85" s="2">
         <v>1085</v>
       </c>
       <c r="D85" t="s">
-        <v>161</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="B86" s="2">
         <v>1086</v>
       </c>
       <c r="D86" t="s">
-        <v>161</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
-        <v>86</v>
+        <v>141</v>
       </c>
       <c r="B87" s="2">
         <v>1087</v>
       </c>
       <c r="D87" t="s">
-        <v>161</v>
+        <v>4</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
-        <v>87</v>
+        <v>142</v>
       </c>
       <c r="B88" s="2">
         <v>1088</v>
@@ -1587,7 +1587,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="B89" s="2">
         <v>1089</v>
@@ -1595,7 +1595,7 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
       <c r="B90" s="2">
         <v>1090</v>
@@ -1603,7 +1603,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="B91" s="2">
         <v>1091</v>
@@ -1611,7 +1611,7 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
       <c r="B92" s="2">
         <v>1092</v>
@@ -1619,7 +1619,7 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>92</v>
+        <v>147</v>
       </c>
       <c r="B93" s="2">
         <v>1093</v>
@@ -1627,7 +1627,7 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="B94" s="2">
         <v>1094</v>
@@ -1635,7 +1635,7 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>94</v>
+        <v>149</v>
       </c>
       <c r="B95" s="2">
         <v>1095</v>
@@ -1643,7 +1643,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="B96" s="2">
         <v>1096</v>
@@ -1651,7 +1651,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>96</v>
+        <v>151</v>
       </c>
       <c r="B97" s="2">
         <v>1097</v>
@@ -1659,7 +1659,7 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="B98" s="2">
         <v>1098</v>
@@ -1667,7 +1667,7 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="B99" s="2">
         <v>1099</v>
@@ -1675,7 +1675,7 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="B100" s="2">
         <v>1100</v>
@@ -1683,7 +1683,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="B101" s="2">
         <v>1101</v>
@@ -1691,7 +1691,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="B102" s="2">
         <v>1102</v>
@@ -1699,7 +1699,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>102</v>
+        <v>153</v>
       </c>
       <c r="B103" s="2">
         <v>1103</v>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>103</v>
+        <v>154</v>
       </c>
       <c r="B104" s="2">
         <v>1104</v>
@@ -1715,7 +1715,7 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>104</v>
+        <v>59</v>
       </c>
       <c r="B105" s="2">
         <v>1105</v>
@@ -1723,7 +1723,7 @@
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>105</v>
+        <v>1</v>
       </c>
       <c r="B106" s="2">
         <v>1106</v>
@@ -1731,7 +1731,7 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>106</v>
+        <v>60</v>
       </c>
       <c r="B107" s="2">
         <v>1107</v>
@@ -1739,7 +1739,7 @@
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="B108" s="2">
         <v>1108</v>
@@ -1747,7 +1747,7 @@
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>108</v>
+        <v>62</v>
       </c>
       <c r="B109" s="2">
         <v>1109</v>
@@ -1755,7 +1755,7 @@
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="B110" s="2">
         <v>1110</v>
@@ -1763,7 +1763,7 @@
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
-        <v>110</v>
+        <v>64</v>
       </c>
       <c r="B111" s="2">
         <v>1111</v>
@@ -1771,7 +1771,7 @@
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
-        <v>111</v>
+        <v>65</v>
       </c>
       <c r="B112" s="2">
         <v>1112</v>
@@ -1779,7 +1779,7 @@
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>112</v>
+        <v>66</v>
       </c>
       <c r="B113" s="2">
         <v>1113</v>
@@ -1787,7 +1787,7 @@
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>113</v>
+        <v>67</v>
       </c>
       <c r="B114" s="2">
         <v>1114</v>
@@ -1795,7 +1795,7 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="B115" s="2">
         <v>1115</v>
@@ -1803,7 +1803,7 @@
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>162</v>
+        <v>107</v>
       </c>
       <c r="B116" s="2">
         <v>11151</v>
@@ -1811,7 +1811,7 @@
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>115</v>
+        <v>69</v>
       </c>
       <c r="B117" s="2">
         <v>1116</v>
@@ -1819,7 +1819,7 @@
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>116</v>
+        <v>70</v>
       </c>
       <c r="B118" s="2">
         <v>1117</v>
@@ -1827,7 +1827,7 @@
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>117</v>
+        <v>71</v>
       </c>
       <c r="B119" s="2">
         <v>1118</v>
@@ -1835,7 +1835,7 @@
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
-        <v>118</v>
+        <v>72</v>
       </c>
       <c r="B120" s="2">
         <v>1119</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="B121" s="2">
         <v>1120</v>
@@ -1851,7 +1851,7 @@
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="B122" s="2">
         <v>1121</v>
@@ -1859,7 +1859,7 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
-        <v>121</v>
+        <v>75</v>
       </c>
       <c r="B123" s="2">
         <v>1122</v>
@@ -1867,7 +1867,7 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="B124" s="2">
         <v>1123</v>
@@ -1875,7 +1875,7 @@
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="B125" s="2">
         <v>1124</v>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
-        <v>124</v>
+        <v>78</v>
       </c>
       <c r="B126" s="2">
         <v>1125</v>
@@ -1891,7 +1891,7 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="B127" s="2">
         <v>1126</v>
@@ -1899,7 +1899,7 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="B128" s="2">
         <v>1127</v>
@@ -1907,7 +1907,7 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>127</v>
+        <v>81</v>
       </c>
       <c r="B129" s="2">
         <v>1128</v>
@@ -1915,7 +1915,7 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="B130" s="2">
         <v>1129</v>
@@ -1923,7 +1923,7 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="B131" s="2">
         <v>1130</v>
@@ -1931,7 +1931,7 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>130</v>
+        <v>82</v>
       </c>
       <c r="B132" s="2">
         <v>1131</v>
@@ -1939,7 +1939,7 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
-        <v>131</v>
+        <v>83</v>
       </c>
       <c r="B133" s="2">
         <v>1132</v>
@@ -1947,7 +1947,7 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>132</v>
+        <v>84</v>
       </c>
       <c r="B134" s="2">
         <v>1133</v>
@@ -1955,7 +1955,7 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>133</v>
+        <v>85</v>
       </c>
       <c r="B135" s="2">
         <v>1134</v>
@@ -1963,18 +1963,18 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="B136" s="2">
         <v>1135</v>
       </c>
       <c r="C136" t="s">
-        <v>163</v>
+        <v>109</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="B137" s="2">
         <v>1136</v>
@@ -1982,7 +1982,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="B138" s="2">
         <v>1137</v>
@@ -1990,7 +1990,7 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="B139" s="2">
         <v>1138</v>
@@ -1998,7 +1998,7 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>138</v>
+        <v>113</v>
       </c>
       <c r="B140" s="2">
         <v>1139</v>
@@ -2006,7 +2006,7 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="B141" s="2">
         <v>1140</v>
@@ -2014,7 +2014,7 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="B142" s="2">
         <v>1141</v>
@@ -2022,7 +2022,7 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="B143" s="2">
         <v>1142</v>
@@ -2030,7 +2030,7 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="B144" s="2">
         <v>1143</v>
@@ -2038,18 +2038,18 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="B145" s="2">
         <v>1144</v>
       </c>
       <c r="C145" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="B146" s="2">
         <v>1145</v>
@@ -2057,7 +2057,7 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>145</v>
+        <v>119</v>
       </c>
       <c r="B147" s="2">
         <v>1146</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
-        <v>146</v>
+        <v>46</v>
       </c>
       <c r="B148" s="2">
         <v>1147</v>
@@ -2073,29 +2073,29 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B149" s="2">
         <v>1148</v>
       </c>
       <c r="C149" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B150" s="2">
         <v>1149</v>
       </c>
       <c r="C150" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
-        <v>149</v>
+        <v>120</v>
       </c>
       <c r="B151" s="2">
         <v>1150</v>
@@ -2103,7 +2103,7 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
-        <v>162</v>
+        <v>107</v>
       </c>
       <c r="B152" s="2">
         <v>1151</v>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
-        <v>150</v>
+        <v>47</v>
       </c>
       <c r="B153" s="2">
         <v>1152</v>
@@ -2119,7 +2119,7 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
-        <v>151</v>
+        <v>48</v>
       </c>
       <c r="B154" s="2">
         <v>1153</v>
@@ -2127,7 +2127,7 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>152</v>
+        <v>49</v>
       </c>
       <c r="B155" s="2">
         <v>1154</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="B156" s="2">
         <v>1155</v>
@@ -2143,7 +2143,7 @@
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>154</v>
+        <v>122</v>
       </c>
       <c r="B157" s="2">
         <v>1156</v>
@@ -2151,7 +2151,7 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>155</v>
+        <v>123</v>
       </c>
       <c r="B158" s="2">
         <v>1157</v>
@@ -2159,18 +2159,18 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B159" s="2">
         <v>1158</v>
       </c>
       <c r="C159" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B160" s="2">
         <v>1159</v>
@@ -2178,7 +2178,7 @@
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B161" s="2">
         <v>1160</v>
@@ -2186,7 +2186,7 @@
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B162" s="2">
         <v>1161</v>

</xml_diff>